<commit_message>
Otro reporte, pero sin vacíos
</commit_message>
<xml_diff>
--- a/Reporte_Radio - copia.xlsx
+++ b/Reporte_Radio - copia.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\ReporteRadio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CF5F0CD-A8E5-445C-8A36-45E62A86B6B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A99C6F-9F8C-4F47-A2C9-6A61023EE9A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5C0A4D95-2E1C-48C6-BF5D-23E5933B5009}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1947" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1955" uniqueCount="336">
   <si>
     <t>Fecha</t>
   </si>
@@ -1047,6 +1047,15 @@
   </si>
   <si>
     <t>En su colaboración semanal, Gustavo Rosales transmite una entrevista realizada a la multimedallista hidalguense Ivana Reyes Palacios, en la categoría de tiro con arco, que, en esta olimpiada nacional dio la sorpresa y consiguió cuatro preseas para el Estado. En la entrevista comentó que, dentro de sus metas está participar en los juegos olímpicos de 2028.</t>
+  </si>
+  <si>
+    <t>Reclutamiento</t>
+  </si>
+  <si>
+    <t>Bibliotecas</t>
+  </si>
+  <si>
+    <t>Transición a Fiscalía</t>
   </si>
 </sst>
 </file>
@@ -1101,10 +1110,7 @@
   </cellStyles>
   <dxfs count="11">
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="d/m/yy;@"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1131,7 +1137,10 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="d/m/yy;@"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1172,20 +1181,20 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{717AF3FA-E95C-4D17-A1C9-B8D7CBE34EF0}" name="Información1" displayName="Información1" ref="A1:M195" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:M195" xr:uid="{717AF3FA-E95C-4D17-A1C9-B8D7CBE34EF0}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{EB19E952-2F9B-4E64-9A19-C7B52F571890}" uniqueName="1" name="Fecha" queryTableFieldId="1" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{A48192A8-75D4-491A-AE26-6A961BCFF6FF}" uniqueName="11" name="Día" queryTableFieldId="11" dataDxfId="0">
+    <tableColumn id="1" xr3:uid="{EB19E952-2F9B-4E64-9A19-C7B52F571890}" uniqueName="1" name="Fecha" queryTableFieldId="1" dataDxfId="10"/>
+    <tableColumn id="11" xr3:uid="{A48192A8-75D4-491A-AE26-6A961BCFF6FF}" uniqueName="11" name="Día" queryTableFieldId="11" dataDxfId="9">
       <calculatedColumnFormula>IF(Información1[[#This Row],[Fecha]]='Ajuste de fechas'!$A$2,"Día actual","Día anterior")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{4F30991B-1882-48AE-BBBC-64FCA8279BA1}" uniqueName="12" name="Radiodifusora" queryTableFieldId="12" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{4F30991B-1882-48AE-BBBC-64FCA8279BA1}" uniqueName="12" name="Radiodifusora" queryTableFieldId="12" dataDxfId="8"/>
     <tableColumn id="13" xr3:uid="{517B0A2C-DF6B-4794-9C97-29B5F886839A}" uniqueName="13" name="Programa" queryTableFieldId="13"/>
-    <tableColumn id="3" xr3:uid="{3DD51BE0-FD5E-43FC-B095-76D2D204B603}" uniqueName="3" name="Titular" queryTableFieldId="3" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{26FEF469-35CF-4C60-A1AE-6CF1039F413A}" uniqueName="6" name="Dependencia" queryTableFieldId="6" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{A1DC7DCD-8016-4C54-B5CE-B9D28C1CC171}" uniqueName="9" name="Tema" queryTableFieldId="9" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{B82BEC87-3598-42A1-B8B9-34F0762C5BB2}" uniqueName="8" name="Canal" queryTableFieldId="8" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{692FF757-1020-40D1-A4F6-D548E7C4E980}" uniqueName="10" name="Estatus" queryTableFieldId="10" dataDxfId="5"/>
-    <tableColumn id="14" xr3:uid="{C39741D3-700F-486E-B020-D2528DDA6016}" uniqueName="14" name="Clasificación" queryTableFieldId="14" dataDxfId="4"/>
-    <tableColumn id="15" xr3:uid="{33A7D71D-EB15-4FD0-8031-4FF610A857BA}" uniqueName="15" name="Autor" queryTableFieldId="15" dataDxfId="3"/>
-    <tableColumn id="16" xr3:uid="{B0698B4E-43A3-42F4-8099-288A9107B833}" uniqueName="16" name="Género" queryTableFieldId="16" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{3DD51BE0-FD5E-43FC-B095-76D2D204B603}" uniqueName="3" name="Titular" queryTableFieldId="3" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{26FEF469-35CF-4C60-A1AE-6CF1039F413A}" uniqueName="6" name="Dependencia" queryTableFieldId="6" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{A1DC7DCD-8016-4C54-B5CE-B9D28C1CC171}" uniqueName="9" name="Tema" queryTableFieldId="9" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{B82BEC87-3598-42A1-B8B9-34F0762C5BB2}" uniqueName="8" name="Canal" queryTableFieldId="8" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{692FF757-1020-40D1-A4F6-D548E7C4E980}" uniqueName="10" name="Estatus" queryTableFieldId="10" dataDxfId="3"/>
+    <tableColumn id="14" xr3:uid="{C39741D3-700F-486E-B020-D2528DDA6016}" uniqueName="14" name="Clasificación" queryTableFieldId="14" dataDxfId="2"/>
+    <tableColumn id="15" xr3:uid="{33A7D71D-EB15-4FD0-8031-4FF610A857BA}" uniqueName="15" name="Autor" queryTableFieldId="15" dataDxfId="1"/>
+    <tableColumn id="16" xr3:uid="{B0698B4E-43A3-42F4-8099-288A9107B833}" uniqueName="16" name="Género" queryTableFieldId="16" dataDxfId="0"/>
     <tableColumn id="17" xr3:uid="{0B5B25B3-3146-48A6-884B-EBAF2D195A97}" uniqueName="17" name="Recuento" queryTableFieldId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2012,6 +2021,9 @@
       <c r="F12" t="s">
         <v>70</v>
       </c>
+      <c r="G12" t="s">
+        <v>133</v>
+      </c>
       <c r="H12" t="s">
         <v>32</v>
       </c>
@@ -2134,6 +2146,9 @@
       </c>
       <c r="F15" t="s">
         <v>21</v>
+      </c>
+      <c r="G15" t="s">
+        <v>117</v>
       </c>
       <c r="H15" t="s">
         <v>32</v>
@@ -6248,6 +6263,9 @@
       <c r="F113" t="s">
         <v>67</v>
       </c>
+      <c r="G113" t="s">
+        <v>335</v>
+      </c>
       <c r="H113" t="s">
         <v>32</v>
       </c>
@@ -6287,6 +6305,9 @@
       <c r="F114" t="s">
         <v>19</v>
       </c>
+      <c r="G114" t="s">
+        <v>304</v>
+      </c>
       <c r="H114" t="s">
         <v>32</v>
       </c>
@@ -6368,6 +6389,9 @@
       <c r="F116" t="s">
         <v>15</v>
       </c>
+      <c r="G116" t="s">
+        <v>334</v>
+      </c>
       <c r="H116" t="s">
         <v>32</v>
       </c>
@@ -6701,6 +6725,9 @@
       <c r="F124" t="s">
         <v>26</v>
       </c>
+      <c r="G124" t="s">
+        <v>277</v>
+      </c>
       <c r="H124" t="s">
         <v>32</v>
       </c>
@@ -7286,6 +7313,9 @@
       <c r="F138" t="s">
         <v>19</v>
       </c>
+      <c r="G138" t="s">
+        <v>333</v>
+      </c>
       <c r="H138" t="s">
         <v>11</v>
       </c>
@@ -7324,6 +7354,9 @@
       </c>
       <c r="F139" t="s">
         <v>24</v>
+      </c>
+      <c r="G139" t="s">
+        <v>333</v>
       </c>
       <c r="H139" t="s">
         <v>11</v>

</xml_diff>